<commit_message>
Fix: Rebuild Cover Sheet with valid Excel format
</commit_message>
<xml_diff>
--- a/projects/cost-data/245-C-AA-001_01_001.xlsx
+++ b/projects/cost-data/245-C-AA-001_01_001.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,30 +29,22 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Aptos Narrow"/>
-      <b val="1"/>
-      <color rgb="001F5C99"/>
-      <sz val="22"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="16"/>
     </font>
     <font>
-      <name val="Aptos Narrow"/>
-      <color rgb="00000000"/>
+      <name val="Calibri"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00000000"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Aptos Narrow"/>
+      <name val="Calibri"/>
       <color rgb="00595959"/>
       <sz val="10"/>
     </font>
@@ -77,22 +69,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -459,76 +448,69 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C4:C17"/>
+  <dimension ref="C10:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="3" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1"/>
-    <row r="2" ht="15" customHeight="1"/>
-    <row r="3" ht="15" customHeight="1"/>
-    <row r="4" ht="20" customHeight="1">
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>◆ CTS Nordics</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1"/>
-    <row r="6" ht="20" customHeight="1"/>
-    <row r="7" ht="20" customHeight="1"/>
-    <row r="8" ht="20" customHeight="1"/>
-    <row r="9" ht="15" customHeight="1"/>
-    <row r="10" ht="22" customHeight="1">
-      <c r="C10" s="2" t="inlineStr">
+    <row r="1" ht="18" customHeight="1"/>
+    <row r="2" ht="18" customHeight="1"/>
+    <row r="3" ht="18" customHeight="1"/>
+    <row r="4" ht="18" customHeight="1"/>
+    <row r="5" ht="18" customHeight="1"/>
+    <row r="6" ht="18" customHeight="1"/>
+    <row r="7" ht="18" customHeight="1"/>
+    <row r="8" ht="18" customHeight="1"/>
+    <row r="9" ht="18" customHeight="1"/>
+    <row r="10" ht="18" customHeight="1">
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>PROJECT DCM103</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1"/>
+    <row r="11" ht="18" customHeight="1"/>
     <row r="12" ht="18" customHeight="1">
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Application for Payment</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1"/>
+    <row r="13" ht="18" customHeight="1"/>
     <row r="14" ht="18" customHeight="1">
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Bulk Data Centers N01 DCM103 AS</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1"/>
-    <row r="16" ht="15" customHeight="1"/>
-    <row r="17" ht="16" customHeight="1">
-      <c r="C17" s="5" t="inlineStr">
+    <row r="15" ht="18" customHeight="1"/>
+    <row r="16" ht="18" customHeight="1"/>
+    <row r="17" ht="18" customHeight="1">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Application for Payment No.01 - Feb 26</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1"/>
-    <row r="19" ht="15" customHeight="1"/>
-    <row r="20" ht="15" customHeight="1"/>
-    <row r="21" ht="15" customHeight="1"/>
-    <row r="22" ht="15" customHeight="1"/>
-    <row r="23" ht="15" customHeight="1"/>
-    <row r="24" ht="15" customHeight="1"/>
+    <row r="18" ht="18" customHeight="1"/>
+    <row r="19" ht="18" customHeight="1"/>
+    <row r="20" ht="18" customHeight="1"/>
+    <row r="21" ht="18" customHeight="1"/>
+    <row r="22" ht="18" customHeight="1"/>
+    <row r="23" ht="18" customHeight="1"/>
+    <row r="24" ht="18" customHeight="1"/>
+    <row r="25" ht="18" customHeight="1"/>
+    <row r="26" ht="18" customHeight="1"/>
+    <row r="27" ht="18" customHeight="1"/>
+    <row r="28" ht="18" customHeight="1"/>
+    <row r="29" ht="18" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9"/>
 </worksheet>
 </file>
 

</xml_diff>